<commit_message>
精简 colors.json 为 v2 schema
</commit_message>
<xml_diff>
--- a/artkal-m-221-official/colors.xlsx
+++ b/artkal-m-221-official/colors.xlsx
@@ -2489,12 +2489,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>原始查询名</t>
+          <t>系列短名</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>优肯418色中的 M221</t>
+          <t>优肯M221色</t>
         </is>
       </c>
     </row>

</xml_diff>